<commit_message>
sync 2026-03-15 14:45 | configs/config_jeans.json,docs/CHECKLIST.md,imagenes/asset_repo/bitly.png,imagenes/asset_repo/link.png,precios/lista_jeans.xlsx
</commit_message>
<xml_diff>
--- a/precios/lista_jeans.xlsx
+++ b/precios/lista_jeans.xlsx
@@ -150,6 +150,31 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <dxfs count="3">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF2A6099"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFFF"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>

</xml_diff>